<commit_message>
:sparkles: Add dual-engine XLSX style showcase outputs
</commit_message>
<xml_diff>
--- a/examples/style_showcase/output.xlsx
+++ b/examples/style_showcase/output.xlsx
@@ -220,32 +220,20 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
       <left style="thick">
         <color rgb="FF1F3864"/>
       </left>
@@ -254,13 +242,8 @@
       <bottom style="thin">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -271,13 +254,8 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -288,13 +266,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -305,13 +278,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -322,13 +290,8 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -339,13 +302,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -356,13 +314,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFDCE6F1"/>
@@ -371,26 +324,16 @@
       <bottom style="thin">
         <color rgb="FFDCE6F1"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
         <color rgb="FFDCE6F1"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFDCE6F1"/>
@@ -399,13 +342,8 @@
         <color rgb="FFDCE6F1"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
-      <start/>
-      <end/>
       <left style="thin">
         <color rgb="FF1F3864"/>
       </left>
@@ -421,8 +359,6 @@
       <diagonal style="medium">
         <color rgb="FF1F3864"/>
       </diagonal>
-      <vertical/>
-      <horizontal/>
     </border>
     <border>
       <start style="thick">
@@ -439,13 +375,8 @@
       <bottom style="thin">
         <color rgb="FF1F3864"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -458,13 +389,8 @@
       <bottom style="medium">
         <color rgb="FFFFFFFF"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -477,9 +403,6 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
     <border>
       <left/>
@@ -602,8 +525,6 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -612,13 +533,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -627,13 +543,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -642,13 +553,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -657,13 +563,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -672,13 +573,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -687,13 +583,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -702,13 +593,8 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -717,26 +603,16 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -745,13 +621,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -760,13 +631,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -775,13 +641,8 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -790,9 +651,6 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
   </borders>
   <cellStyleXfs count="1">

</xml_diff>

<commit_message>
⚡ Enhance PDF and XLSX rendering with new fast paths and tests (#12)
Co-authored-by: Joel Samraj <joelsamrajs@gmail.com>
</commit_message>
<xml_diff>
--- a/examples/style_showcase/output.xlsx
+++ b/examples/style_showcase/output.xlsx
@@ -220,32 +220,20 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
       <left style="thick">
         <color rgb="FF1F3864"/>
       </left>
@@ -254,13 +242,8 @@
       <bottom style="thin">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -271,13 +254,8 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -288,13 +266,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -305,13 +278,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -322,13 +290,8 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -339,13 +302,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -356,13 +314,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFDCE6F1"/>
@@ -371,26 +324,16 @@
       <bottom style="thin">
         <color rgb="FFDCE6F1"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
         <color rgb="FFDCE6F1"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFDCE6F1"/>
@@ -399,13 +342,8 @@
         <color rgb="FFDCE6F1"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
     <border diagonalUp="1" diagonalDown="1">
-      <start/>
-      <end/>
       <left style="thin">
         <color rgb="FF1F3864"/>
       </left>
@@ -421,8 +359,6 @@
       <diagonal style="medium">
         <color rgb="FF1F3864"/>
       </diagonal>
-      <vertical/>
-      <horizontal/>
     </border>
     <border>
       <start style="thick">
@@ -439,13 +375,8 @@
       <bottom style="thin">
         <color rgb="FF1F3864"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -458,13 +389,8 @@
       <bottom style="medium">
         <color rgb="FFFFFFFF"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -477,9 +403,6 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
     <border>
       <left/>
@@ -602,8 +525,6 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -612,13 +533,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -627,13 +543,8 @@
       <bottom style="medium">
         <color rgb="FFC55A11"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -642,13 +553,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -657,13 +563,8 @@
       <bottom style="medium">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -672,13 +573,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -687,13 +583,8 @@
         <color rgb="FF2E75B6"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -702,13 +593,8 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -717,26 +603,16 @@
         <color rgb="FF375623"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
         <color rgb="FF2E75B6"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -745,13 +621,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -760,13 +631,8 @@
         <color rgb="FFC55A11"/>
       </top>
       <bottom/>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -775,13 +641,8 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
-    </border>
-    <border>
-      <start/>
-      <end/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FFFFFFFF"/>
@@ -790,9 +651,6 @@
       <bottom style="medium">
         <color rgb="FF375623"/>
       </bottom>
-      <diagonal/>
-      <vertical/>
-      <horizontal/>
     </border>
   </borders>
   <cellStyleXfs count="1">

</xml_diff>